<commit_message>
Asset status: demo assets follow the real fault log; show real faults and spares
The demo seed now lists an asset only where the iSMM fault log (1 Aug to 20 Oct
2026) records faults on that kind of equipment in that building, named by its
iSMM tag where the remarks give one (CD-AHU-07, AHU-CM-10, CM-F-L1, LG-OG-4...).
Unbacked assets are removed (dome chillers, water play pump, wetland pump,
plaza lift, Floral Clock DB, kiosk outlets) and the demo story moves onto real
equipment. States and readings stay synthetic.

Each asset page shows the matching fault records and the spares held for it
(Ref. ID, store, quantity) when GBB_DATA_DIR is set. A seed rebuild now drops
assets the seed no longer lists. "Fleet status" is renamed "Asset status".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05_Current_Prototype/data/examples/site/electrical-bad-sample.xlsx
+++ b/05_Current_Prototype/data/examples/site/electrical-bad-sample.xlsx
@@ -481,7 +481,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EMS-FDMCHL01</t>
+          <t>EMS-FDMAHU01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -506,7 +506,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EMS-FDMCHL01</t>
+          <t>EMS-FDMAHU01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>91.59999999999999</v>
+        <v>25.7</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -531,7 +531,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EMS-FDMCHL01</t>
+          <t>EMS-FDMAHU01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>32.99</v>
+        <v>9.26</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -556,7 +556,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EMS-FDMCHL01</t>
+          <t>EMS-FDMAHU01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>45881.42</v>
+        <v>45875.49</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -581,7 +581,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EMS-FDMCHL01</t>
+          <t>EMS-FDMAHU01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EMS-FDMCHL01</t>
+          <t>EMS-FDMAHU01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -916,7 +916,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EMS-FDMCHL01</t>
+          <t>EMS-FDMAHU01</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">

</xml_diff>